<commit_message>
Fix uiwindow UILayer and UIAnimationType values for JulyCore enums.
Use Normal(100)/Popup(200) layers and Scale(3) enter/exit animation for window panels.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Tools/Luban/DataTables/Datas/CozyYard/uiwindow.xlsx
+++ b/Tools/Luban/DataTables/Datas/CozyYard/uiwindow.xlsx
@@ -643,7 +643,7 @@
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
@@ -668,16 +668,16 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I5" t="b">
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6">
@@ -702,16 +702,16 @@
         <v>1</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I6" t="b">
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="7">
@@ -736,16 +736,16 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I7" t="b">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="8">
@@ -770,16 +770,16 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I8" t="b">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="9">
@@ -804,16 +804,16 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I9" t="b">
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="10">
@@ -838,16 +838,16 @@
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I10" t="b">
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="11">
@@ -872,16 +872,16 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I11" t="b">
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12">
@@ -906,16 +906,16 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I12" t="b">
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
     <row r="13">
@@ -940,16 +940,16 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I13" t="b">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>2</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>